<commit_message>
rename ENS -> HOWE (Hockey Outcomes via Weighted Ensemble); canonical howe.py
Pure rebrand of the prereg'd ensemble (PLAN_V4 I3 @ 64baf45): math, params, seeds
unchanged — report4 rerun after the rename reproduced all projections CSVs
byte-identically. Locked prereg text in PLAN_*/NOTES history keeps the original
"ENS" wording as the historical record.

Refactor: new src/howe.py is the single canonical rebuild of the deterministic
HOWE 2026-27 sim (ratings + rebuild_sim), replacing duplicated copies in
price_milestones.py and optimize_full100.py; optimize_board.py imports from it.
Renamed artifacts: projections_*_ens.csv -> *_howe.csv, rating_ens -> rating_howe,
model_ens -> model_howe, ens_restatement -> howe_restatement, xlsx sheets ENS ->
HOWE, live.py model key "ens" -> "howe". milestones_vs_model.csv refreshed (board
lines added after the last pricing run; all previously committed rows unchanged).
README added. Battery 68/68; live parity 0.000000 Elo.
</commit_message>
<xml_diff>
--- a/output/nhl_2026_27_projections_v4.xlsx
+++ b/output/nhl_2026_27_projections_v4.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Projections_2026_27_ENS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Projections_2026_27_HOWE" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Projections_2026_27_v4" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Projections_2027_28_ENS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Projections_2027_28_HOWE" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Projections_2027_28_v4" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Market_vs_Model" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Prospect_Pipeline" sheetId="7" state="visible" r:id="rId7"/>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,67 +466,74 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CO-HEADLINES: Projections_2026_27_ENS (locked 50/50 v1+v4 ensemble) and _v4.</t>
+          <t>CO-HEADLINES: Projections_2026_27_HOWE (locked 50/50 v1+v4 ensemble) and _v4.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>The live 2026-27 season scores v1, v4 and ENS — pre-registered holdout.</t>
+          <t>HOWE = Hockey Outcomes via Weighted Ensemble (prereg name ENS; renamed 2026-08-19, math/seeds unchanged).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>The live 2026-27 season scores v1, v4 and HOWE — pre-registered holdout.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Gated in this round (train-only, 2018-2026 untouched):</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1. GOALIE GAME LAYER: starter rotation per game, b2b backup rule (beta_b2b=0.5 declared), zero-mean (verified 0.002 pts). GATE G PASS (coverage 0.861).</t>
+          <t>Gated in this round (train-only, 2018-2026 untouched):</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2. AVAILABILITY 2.0: + zero-GP mass (P0 up to 14.6% at 36+), goalie G1 slot, h2 ages. GATE A2 PASS (coverage 0.872, spread 0.133 vs bound 0.117+0.02 — passes by 0.004, watch live). Persistence DROPPED (EB lost to bucket-only).</t>
+          <t>1. GOALIE GAME LAYER: starter rotation per game, b2b backup rule (beta_b2b=0.5 declared), zero-mean (verified 0.002 pts). GATE G PASS (coverage 0.861).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3. PROSPECT PIPELINE: draft-&gt;panel join (98% on picks 1-15), train ramps; GATE F2: h1 dMAE -0.0065, h2 -0.1338 (largest single train gain since v2), sign-stable 1.00 — ENTERS both horizons.</t>
+          <t>2. AVAILABILITY 2.0: + zero-GP mass (P0 up to 14.6% at 36+), goalie G1 slot, h2 ages. GATE A2 PASS (coverage 0.872, spread 0.133 vs bound 0.117+0.02 — passes by 0.004, watch live). Persistence DROPPED (EB lost to bucket-only).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4. OVERLAY AMENDED + REPRODUCIBLE: rho spec-robust 0.843 with production-consistent weights -&gt; rho*=0.421 (v3.1's 1.011 reproduced; its gain was the intercept fixing a weighting artifact, not the selection control).</t>
+          <t>3. PROSPECT PIPELINE: draft-&gt;panel join (98% on picks 1-15), train ramps; GATE F2: h1 dMAE -0.0065, h2 -0.1338 (largest single train gain since v2), sign-stable 1.00 — ENTERS both horizons.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>4. OVERLAY AMENDED + REPRODUCIBLE: rho spec-robust 0.843 with production-consistent weights -&gt; rho*=0.421 (v3.1's 1.011 reproduced; its gain was the intercept fixing a weighting artifact, not the selection control).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>5. BUGS: float64 tiebreak key restores ROW (+W added); b2b constant 38 reproduced from committed code (t -5.3/+6.7); live.py rebuilt to the validated estimator with full odds output.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Market_vs_Model: user-recorded Cup board 2026-08-17 (overround 1.255). Fair odds are break-even prices, NOT bet instructions; see the stake column for quarter-Kelly at actual prices — it is deliberately tiny.</t>
         </is>
@@ -10111,7 +10118,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>model_ens</t>
+          <t>model_howe</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">

</xml_diff>